<commit_message>
Update - Full Logs Added - Variables Not Used Deleted - Activities Names Changed
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELLCI5\Documents\UiPath\Dermalogica_InternetPriceMonitoring\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9D45066-4E66-41A7-8378-E40315F4612D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6043687-2A74-403C-ABB6-CEBA55132957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23929" yWindow="-113" windowWidth="16253" windowHeight="12322" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
   <si>
     <t>Name</t>
   </si>
@@ -149,6 +149,12 @@
   </si>
   <si>
     <t>C:\Users\DELLCI5\Downloads\RPA_InternetPriceMonitoring_Report.xlsx</t>
+  </si>
+  <si>
+    <t>Websites_Path</t>
+  </si>
+  <si>
+    <t>Data\Websites.xlsx</t>
   </si>
 </sst>
 </file>
@@ -596,7 +602,14 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Update - All CloseApps Applied, Browser Never Closes - Asset Added - Dynamic Dictionary
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELLCI5\Documents\UiPath\Dermalogica_InternetPriceMonitoring\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6043687-2A74-403C-ABB6-CEBA55132957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E408CE0D-9C08-4ABC-B79B-5A178503B94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23929" yWindow="-113" windowWidth="16253" windowHeight="12322" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23929" yWindow="-113" windowWidth="16253" windowHeight="12322" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
   <si>
     <t>Name</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>Data\Websites.xlsx</t>
+  </si>
+  <si>
+    <t>DermalogicaPricesExtracting</t>
   </si>
 </sst>
 </file>
@@ -2814,7 +2817,17 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Update - Exceptions fully added - Assets implemented
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELLCI5\Documents\UiPath\Dermalogica_InternetPriceMonitoring\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E408CE0D-9C08-4ABC-B79B-5A178503B94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA595D9D-4B0B-482E-90D1-2A82B6184120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23929" yWindow="-113" windowWidth="16253" windowHeight="12322" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
   <si>
     <t>Name</t>
   </si>
@@ -158,6 +158,18 @@
   </si>
   <si>
     <t>DermalogicaPricesExtracting</t>
+  </si>
+  <si>
+    <t>Mail_Receiver</t>
+  </si>
+  <si>
+    <t>Output_Folder</t>
+  </si>
+  <si>
+    <t>Retries_Webpage</t>
+  </si>
+  <si>
+    <t>ExcelProgram_Path</t>
   </si>
 </sst>
 </file>
@@ -2828,10 +2840,50 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Update - Check app state corrected - Structure Fully Enhanced
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELLCI5\Documents\UiPath\Dermalogica_InternetPriceMonitoring\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA595D9D-4B0B-482E-90D1-2A82B6184120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FD3E7B-7523-4A8A-81A1-CBC426034E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>Name</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>ExcelProgram_Path</t>
+  </si>
+  <si>
+    <t>Copies_Path</t>
   </si>
 </sst>
 </file>
@@ -2884,7 +2887,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>